<commit_message>
sprint 5 kelar, fokus upload
</commit_message>
<xml_diff>
--- a/sprint_plan.xlsx
+++ b/sprint_plan.xlsx
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Per tanggal 20 June 2026 · Tim 1 developer</t>
+          <t>Per tanggal 05 July 2026 · Tim 1 developer</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>MVP (Minimum Viable Product) — sudah berjalan untuk uji coba internal</t>
+          <t>Beta — 3 dari 6 sprint sudah selesai. Aplikasi sudah lengkap untuk pemakaian internal.</t>
         </is>
       </c>
     </row>
@@ -881,19 +881,19 @@
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Subtitle Otomatis &amp; AI (ringkasan rapat, terjemahan langsung)</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Belum</t>
+          <t>Penyempurnaan Chat &amp; Webinar (Sprint 5: file, reply, pin, typing, read, GIF, soundboard, webinar)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Aplikasi Mobile (Android/iOS)</t>
+          <t>Subtitle Otomatis &amp; AI (Sprint 3: ringkasan rapat, terjemahan langsung)</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -905,7 +905,7 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Peluncuran ke Produksi (live di internet)</t>
+          <t>Aplikasi Mobile (Sprint 4: Android/iOS + PWA)</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -914,28 +914,40 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="8" customHeight="1"/>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Peluncuran ke Produksi (Sprint 6: live di internet)</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="8" customHeight="1"/>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Keterangan Status</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Selesai = sudah berjalan dan bisa digunakan   ·   Berjalan = sedang dikerjakan   ·   Belum = belum dimulai</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 1 dan Sprint 2 sudah tuntas. Aplikasi sekarang punya fitur visual modern setara Zoom: background blur/ganti gambar, peredam bising, timer bicara per peserta, dan ruang pribadi permanen. Sprint berikutnya fokus ke fitur AI: subtitle otomatis selama meeting + ringkasan rapat otomatis.</t>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 1, 2, dan 5 sudah tuntas. Aplikasi sekarang punya fitur chat setara Slack (file upload, reply, pin, typing, read receipts) + mode webinar untuk training internal. Sisa 3 sprint: AI subtitle (butuh anggaran), mobile app, dan peluncuran produksi.</t>
         </is>
       </c>
     </row>
@@ -956,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1308,12 +1320,12 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>Ruang Pribadi (Personal Meeting Room)</t>
+          <t>Mode Webinar</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>Link permanen per pengguna untuk meeting dadakan, otomatis dibuat saat pertama dibuka, tampil di dashboard</t>
+          <t>Ruang hanya boleh diomongin oleh host + cohost. Audiens cuma nonton + chat + reaksi. Cocok untuk training atau kelas online.</t>
         </is>
       </c>
     </row>
@@ -1325,12 +1337,12 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Undangan via Kalender</t>
+          <t>Ruang Pribadi (Personal Meeting Room)</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Otomatis generate file undangan (.ics) untuk Google Calendar / Outlook</t>
+          <t>Link permanen per pengguna untuk meeting dadakan, otomatis dibuat saat pertama dibuka, tampil di dashboard</t>
         </is>
       </c>
     </row>
@@ -1342,1505 +1354,1531 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
+          <t>Undangan via Kalender</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Otomatis generate file undangan (.ics) untuk Google Calendar / Outlook</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
           <t>Undangan via Email</t>
         </is>
       </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>Buka client email dengan template undangan yang sudah berisi link</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="10" customHeight="1"/>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="29" ht="10" customHeight="1"/>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>3. Pengalaman dalam Meeting</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Nama Fitur</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Penjelasan</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Video call multi-peserta</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>Banyak orang bisa video call bersamaan dalam satu ruang</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>Audio dan video jernih</t>
         </is>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
         <is>
           <t>Kualitas audio video adaptif menyesuaikan kecepatan internet</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="32" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Berbagi layar</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>Tampilkan layar komputer ke semua peserta (dengan opsi audio untuk tab)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="15" t="inlineStr">
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>Nyalakan/matikan mic</t>
         </is>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>Tombol toggle mikrofon sendiri kapan saja</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="32" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Nyalakan/matikan kamera</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
         <is>
           <t>Tombol toggle kamera sendiri kapan saja</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="15" t="inlineStr">
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Layar persiapan</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>Sebelum masuk meeting, pengguna bisa preview kamera, atur mic &amp; speaker</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Pilih perangkat</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>Pilih kamera, mic, atau speaker mana yang mau dipakai</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="15" t="inlineStr">
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Background blur kamera</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C39" s="17" t="inlineStr">
         <is>
           <t>Latar belakang otomatis di-blur agar peserta lain fokus ke wajah, bukan ke kamar yang berantakan</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="12" t="inlineStr">
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>Background virtual (4 preset)</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>Ganti latar belakang dengan foto: Kantor, Perpustakaan, Pantai, atau Kafe</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
         <is>
           <t>Peredam bising mikrofon</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="C41" s="17" t="inlineStr">
         <is>
           <t>Otomatis menghilangkan suara latar (ketikan keyboard, kipas, anak menangis) dari mikrofon — pakai teknologi Krisp</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Pin peserta favorit</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>Kunci satu peserta jadi tampilan utama di layar kita saja (lokal, tidak mempengaruhi peserta lain)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="15" t="inlineStr">
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B43" s="16" t="inlineStr">
         <is>
           <t>Timer waktu bicara per peserta</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>Otomatis hitung total waktu bicara tiap peserta, tampil di daftar peserta</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="32" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Mode hemat data</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>Matikan video peserta lain untuk hemat kuota / internet pelan</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="32" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B45" s="16" t="inlineStr">
         <is>
           <t>Picture-in-Picture</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C45" s="17" t="inlineStr">
         <is>
           <t>Video melayang kecil saat pindah tab</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="32" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>Layar penuh</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>Mode fullscreen untuk fokus presentasi</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="32" customHeight="1">
-      <c r="A46" s="15" t="inlineStr">
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Mode Mirror</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr">
+      <c r="C47" s="17" t="inlineStr">
         <is>
           <t>Self-view seperti cermin (default), atau matikan jika diperlukan</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="32" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>Floating self-view</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>Tampilan diri sendiri bisa di-drag bebas atau dikembalikan ke grid</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="10" customHeight="1"/>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
+    <row r="49" ht="10" customHeight="1"/>
+    <row r="50" ht="26" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>4. Kontrol untuk Host (Penyelenggara)</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>Nama Fitur</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>Penjelasan</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="32" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>Sorotkan peserta</t>
         </is>
       </c>
-      <c r="C51" s="14" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
         <is>
           <t>Pin peserta tertentu jadi tampilan besar untuk semua orang</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="32" customHeight="1">
-      <c r="A52" s="15" t="inlineStr">
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B52" s="16" t="inlineStr">
+      <c r="B53" s="16" t="inlineStr">
         <is>
           <t>Bisukan peserta</t>
         </is>
       </c>
-      <c r="C52" s="17" t="inlineStr">
+      <c r="C53" s="17" t="inlineStr">
         <is>
           <t>Mute mikrofon peserta tertentu</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>Matikan kamera peserta</t>
         </is>
       </c>
-      <c r="C53" s="14" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>Force off kamera peserta dari sisi host</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="32" customHeight="1">
-      <c r="A54" s="15" t="inlineStr">
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B54" s="16" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>Hentikan share layar peserta</t>
         </is>
       </c>
-      <c r="C54" s="17" t="inlineStr">
+      <c r="C55" s="17" t="inlineStr">
         <is>
           <t>Stop share layar yang lagi dilakukan peserta</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="32" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>Keluarkan peserta</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr">
+      <c r="C56" s="14" t="inlineStr">
         <is>
           <t>Kick peserta yang mengganggu dari ruang</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="32" customHeight="1">
-      <c r="A56" s="15" t="inlineStr">
+    <row r="57" ht="32" customHeight="1">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B56" s="16" t="inlineStr">
+      <c r="B57" s="16" t="inlineStr">
         <is>
           <t>Bisu semua peserta</t>
         </is>
       </c>
-      <c r="C56" s="17" t="inlineStr">
+      <c r="C57" s="17" t="inlineStr">
         <is>
           <t>Satu klik untuk mute semua orang</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="32" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="12" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>Kunci ruang</t>
         </is>
       </c>
-      <c r="C57" s="14" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>Tidak ada peserta baru yang bisa masuk</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="32" customHeight="1">
-      <c r="A58" s="15" t="inlineStr">
+    <row r="59" ht="32" customHeight="1">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B58" s="16" t="inlineStr">
+      <c r="B59" s="16" t="inlineStr">
         <is>
           <t>Co-host (pendamping host)</t>
         </is>
       </c>
-      <c r="C58" s="17" t="inlineStr">
+      <c r="C59" s="17" t="inlineStr">
         <is>
           <t>Beri akses host ke peserta lain agar bisa membantu mengatur</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="32" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="60" ht="32" customHeight="1">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>Setujui / tolak ruang tunggu</t>
         </is>
       </c>
-      <c r="C59" s="14" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>Saring peserta yang minta masuk ruang</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="32" customHeight="1">
-      <c r="A60" s="15" t="inlineStr">
+    <row r="61" ht="32" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B60" s="16" t="inlineStr">
+      <c r="B61" s="16" t="inlineStr">
         <is>
           <t>Kunci copy chat</t>
         </is>
       </c>
-      <c r="C60" s="17" t="inlineStr">
+      <c r="C61" s="17" t="inlineStr">
         <is>
           <t>Cegah peserta menyalin isi chat</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="32" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="62" ht="32" customHeight="1">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>Matikan chat</t>
         </is>
       </c>
-      <c r="C61" s="14" t="inlineStr">
+      <c r="C62" s="14" t="inlineStr">
         <is>
           <t>Stop chat selama meeting</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="32" customHeight="1">
-      <c r="A62" s="15" t="inlineStr">
+    <row r="63" ht="32" customHeight="1">
+      <c r="A63" s="15" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B62" s="16" t="inlineStr">
+      <c r="B63" s="16" t="inlineStr">
         <is>
           <t>Kunci unmute</t>
         </is>
       </c>
-      <c r="C62" s="17" t="inlineStr">
+      <c r="C63" s="17" t="inlineStr">
         <is>
           <t>Peserta tidak bisa nyalakan mic sendiri (anti-distraksi)</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="32" customHeight="1">
-      <c r="A63" s="12" t="inlineStr">
+    <row r="64" ht="32" customHeight="1">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>Turunkan semua tangan</t>
         </is>
       </c>
-      <c r="C63" s="14" t="inlineStr">
+      <c r="C64" s="14" t="inlineStr">
         <is>
           <t>Reset semua peserta yang angkat tangan sekaligus</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="32" customHeight="1">
-      <c r="A64" s="15" t="inlineStr">
+    <row r="65" ht="32" customHeight="1">
+      <c r="A65" s="15" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B64" s="16" t="inlineStr">
+      <c r="B65" s="16" t="inlineStr">
         <is>
           <t>Reset semua vote</t>
         </is>
       </c>
-      <c r="C64" s="17" t="inlineStr">
+      <c r="C65" s="17" t="inlineStr">
         <is>
           <t>Hapus semua suara Setuju/Tolak</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="32" customHeight="1">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="66" ht="32" customHeight="1">
+      <c r="A66" s="12" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>Jawab / tolak pertanyaan Q&amp;A</t>
         </is>
       </c>
-      <c r="C65" s="14" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>Host bisa jawab pertanyaan dari panel Q&amp;A dengan teks, atau tolak (dismiss)</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="10" customHeight="1"/>
-    <row r="67" ht="26" customHeight="1">
-      <c r="A67" s="11" t="inlineStr">
+    <row r="67" ht="32" customHeight="1">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Pin pesan chat penting</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="inlineStr">
+        <is>
+          <t>Tandai pesan tertentu agar muncul sticky di atas untuk semua orang, klik untuk lompat ke lokasi asli</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="10" customHeight="1"/>
+    <row r="69" ht="26" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>5. Kolaborasi dalam Meeting</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>Nama Fitur</t>
         </is>
       </c>
-      <c r="C68" s="8" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>Penjelasan</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="32" customHeight="1">
-      <c r="A69" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>Chat real-time</t>
-        </is>
-      </c>
-      <c r="C69" s="14" t="inlineStr">
-        <is>
-          <t>Kirim pesan teks ke semua peserta</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="32" customHeight="1">
-      <c r="A70" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B70" s="16" t="inlineStr">
-        <is>
-          <t>Direct Message (DM)</t>
-        </is>
-      </c>
-      <c r="C70" s="17" t="inlineStr">
-        <is>
-          <t>Chat pribadi antara dua peserta saja</t>
         </is>
       </c>
     </row>
     <row r="71" ht="32" customHeight="1">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>Mention pengguna</t>
+          <t>Chat real-time</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>Tag orang dengan @nama</t>
+          <t>Kirim pesan teks ke semua peserta</t>
         </is>
       </c>
     </row>
     <row r="72" ht="32" customHeight="1">
       <c r="A72" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>Edit / hapus pesan</t>
+          <t>Direct Message (DM)</t>
         </is>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
-          <t>Pesan sendiri bisa diedit atau dihapus</t>
+          <t>Chat pribadi antara dua peserta saja</t>
         </is>
       </c>
     </row>
     <row r="73" ht="32" customHeight="1">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>Emoji reactions di pesan</t>
+          <t>Upload file di chat</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
         <is>
-          <t>Reaksi 👍 ❤️ 😂 dll pada tiap pesan</t>
+          <t>Kirim gambar, PDF, dokumen Word/Excel/PowerPoint, atau CSV sampai 10 MB</t>
         </is>
       </c>
     </row>
     <row r="74" ht="32" customHeight="1">
       <c r="A74" s="15" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>Pemilih emoji untuk pesan</t>
+          <t>Kirim GIF</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>Picker dengan banyak emoji standar</t>
+          <t>Cari GIF dari Giphy + kirim langsung ke chat</t>
         </is>
       </c>
     </row>
     <row r="75" ht="32" customHeight="1">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>Notifikasi browser</t>
+          <t>Balas pesan (Reply)</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Notifikasi sistem saat ada chat baru dan tab tidak aktif</t>
+          <t>Balas pesan tertentu dengan kutipan, mirip WhatsApp/Slack</t>
         </is>
       </c>
     </row>
     <row r="76" ht="32" customHeight="1">
       <c r="A76" s="15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B76" s="16" t="inlineStr">
         <is>
-          <t>Toast notifikasi chat</t>
+          <t>Indikator 'sedang mengetik'</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
-          <t>Pop-up kecil saat ada pesan masuk</t>
+          <t>Muncul tulisan 'Andi sedang mengetik...' saat lawan bicara mengetik</t>
         </is>
       </c>
     </row>
     <row r="77" ht="32" customHeight="1">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>Whiteboard digital</t>
+          <t>Centang 'sudah dibaca' di DM</t>
         </is>
       </c>
       <c r="C77" s="14" t="inlineStr">
         <is>
-          <t>Papan tulis kolaboratif, semua peserta bisa menggambar</t>
+          <t>Status pesan ✓ (terkirim) atau ✓✓ (sudah dibaca) di DM</t>
         </is>
       </c>
     </row>
     <row r="78" ht="32" customHeight="1">
       <c r="A78" s="15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B78" s="16" t="inlineStr">
         <is>
-          <t>Anotasi di layar</t>
+          <t>Soundboard efek suara</t>
         </is>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
-          <t>Gambar/tulis langsung di atas video atau share layar</t>
+          <t>Panel dengan 8 efek suara (Tepuk tangan, Drumroll, Airhorn, dll) yang bisa dimainkan ke semua peserta</t>
         </is>
       </c>
     </row>
     <row r="79" ht="32" customHeight="1">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>Polling / vote terstruktur</t>
+          <t>Mention pengguna</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Buat pertanyaan dengan pilihan ganda, peserta vote, hasil terlihat langsung</t>
+          <t>Tag orang dengan @nama</t>
         </is>
       </c>
     </row>
     <row r="80" ht="32" customHeight="1">
       <c r="A80" s="15" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B80" s="16" t="inlineStr">
         <is>
-          <t>Panel Tanya-Jawab (Q&amp;A)</t>
+          <t>Edit / hapus pesan</t>
         </is>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
-          <t>Panel terpisah dari chat: pertanyaan ke host bisa di-vote, host bisa jawab atau dismiss</t>
+          <t>Pesan sendiri bisa diedit atau dihapus</t>
         </is>
       </c>
     </row>
     <row r="81" ht="32" customHeight="1">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
-          <t>Ruang breakout</t>
+          <t>Emoji reactions di pesan</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
         <is>
-          <t>Pisah peserta jadi kelompok-kelompok kecil untuk diskusi</t>
+          <t>Reaksi 👍 ❤️ 😂 dll pada tiap pesan</t>
         </is>
       </c>
     </row>
     <row r="82" ht="32" customHeight="1">
       <c r="A82" s="15" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B82" s="16" t="inlineStr">
         <is>
-          <t>Angkat tangan</t>
+          <t>Pemilih emoji untuk pesan</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
-          <t>Notifikasi visual kalau peserta ingin bicara</t>
+          <t>Picker dengan banyak emoji standar</t>
         </is>
       </c>
     </row>
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>Antrian angkat tangan (FIFO)</t>
+          <t>Notifikasi browser</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>Tampilkan urutan #1, #2, #3 — peserta yang angkat duluan terlihat lebih dulu</t>
+          <t>Notifikasi sistem saat ada chat baru dan tab tidak aktif</t>
         </is>
       </c>
     </row>
     <row r="84" ht="32" customHeight="1">
       <c r="A84" s="15" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B84" s="16" t="inlineStr">
         <is>
-          <t>Vote cepat Setuju/Tolak</t>
+          <t>Toast notifikasi chat</t>
         </is>
       </c>
       <c r="C84" s="17" t="inlineStr">
         <is>
-          <t>Voting hijau/merah instan tanpa perlu polling</t>
+          <t>Pop-up kecil saat ada pesan masuk</t>
         </is>
       </c>
     </row>
     <row r="85" ht="32" customHeight="1">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
-          <t>Reaksi emoji terbang</t>
+          <t>Whiteboard digital</t>
         </is>
       </c>
       <c r="C85" s="14" t="inlineStr">
         <is>
-          <t>👍 ❤️ 🎉 terbang di layar untuk semua orang</t>
+          <t>Papan tulis kolaboratif, semua peserta bisa menggambar</t>
         </is>
       </c>
     </row>
     <row r="86" ht="32" customHeight="1">
       <c r="A86" s="15" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B86" s="16" t="inlineStr">
         <is>
-          <t>Push-to-talk (PTT)</t>
+          <t>Anotasi di layar</t>
         </is>
       </c>
       <c r="C86" s="17" t="inlineStr">
         <is>
-          <t>Tahan spasi untuk bicara, lepas untuk mute lagi</t>
+          <t>Gambar/tulis langsung di atas video atau share layar</t>
         </is>
       </c>
     </row>
     <row r="87" ht="32" customHeight="1">
       <c r="A87" s="12" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>Polling / vote terstruktur</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>Buat pertanyaan dengan pilihan ganda, peserta vote, hasil terlihat langsung</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="32" customHeight="1">
+      <c r="A88" s="15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B88" s="16" t="inlineStr">
+        <is>
+          <t>Panel Tanya-Jawab (Q&amp;A)</t>
+        </is>
+      </c>
+      <c r="C88" s="17" t="inlineStr">
+        <is>
+          <t>Panel terpisah dari chat: pertanyaan ke host bisa di-vote, host bisa jawab atau dismiss</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="32" customHeight="1">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B87" s="13" t="inlineStr">
-        <is>
-          <t>Laser pointer</t>
-        </is>
-      </c>
-      <c r="C87" s="14" t="inlineStr">
-        <is>
-          <t>Cursor laser merah saat presentasi</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="10" customHeight="1"/>
-    <row r="89" ht="26" customHeight="1">
-      <c r="A89" s="11" t="inlineStr">
-        <is>
-          <t>6. Perekaman &amp; Pencatatan</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="22" customHeight="1">
-      <c r="A90" s="8" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>Nama Fitur</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
-          <t>Penjelasan</t>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>Ruang breakout</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Pisah peserta jadi kelompok-kelompok kecil untuk diskusi</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="32" customHeight="1">
+      <c r="A90" s="15" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>Angkat tangan</t>
+        </is>
+      </c>
+      <c r="C90" s="17" t="inlineStr">
+        <is>
+          <t>Notifikasi visual kalau peserta ingin bicara</t>
         </is>
       </c>
     </row>
     <row r="91" ht="32" customHeight="1">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
-          <t>Rekaman meeting</t>
+          <t>Antrian angkat tangan (FIFO)</t>
         </is>
       </c>
       <c r="C91" s="14" t="inlineStr">
         <is>
-          <t>Rekam video meeting otomatis di sisi server</t>
+          <t>Tampilkan urutan #1, #2, #3 — peserta yang angkat duluan terlihat lebih dulu</t>
         </is>
       </c>
     </row>
     <row r="92" ht="32" customHeight="1">
       <c r="A92" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B92" s="16" t="inlineStr">
         <is>
-          <t>Pilih layout rekaman</t>
+          <t>Vote cepat Setuju/Tolak</t>
         </is>
       </c>
       <c r="C92" s="17" t="inlineStr">
         <is>
-          <t>Pilih tampilan: grid, fokus speaker, atau solo speaker</t>
+          <t>Voting hijau/merah instan tanpa perlu polling</t>
         </is>
       </c>
     </row>
     <row r="93" ht="32" customHeight="1">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B93" s="13" t="inlineStr">
         <is>
-          <t>Daftar rekaman</t>
+          <t>Reaksi emoji terbang</t>
         </is>
       </c>
       <c r="C93" s="14" t="inlineStr">
         <is>
-          <t>Lihat semua rekaman per ruang, status, dan ukuran file</t>
+          <t>👍 ❤️ 🎉 terbang di layar untuk semua orang</t>
         </is>
       </c>
     </row>
     <row r="94" ht="32" customHeight="1">
       <c r="A94" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B94" s="16" t="inlineStr">
         <is>
-          <t>Unduh rekaman</t>
+          <t>Push-to-talk (PTT)</t>
         </is>
       </c>
       <c r="C94" s="17" t="inlineStr">
         <is>
-          <t>Link download untuk rekaman yang sudah selesai</t>
+          <t>Tahan spasi untuk bicara, lepas untuk mute lagi</t>
         </is>
       </c>
     </row>
     <row r="95" ht="32" customHeight="1">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>Indikator merekam</t>
+          <t>Laser pointer</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>Badge merah berkedip saat rekaman aktif</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="32" customHeight="1">
-      <c r="A96" s="15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B96" s="16" t="inlineStr">
-        <is>
-          <t>Banner persetujuan rekam</t>
-        </is>
-      </c>
-      <c r="C96" s="17" t="inlineStr">
-        <is>
-          <t>Notifikasi besar muncul sekali saat rekaman dimulai (untuk consent)</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="32" customHeight="1">
-      <c r="A97" s="12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>Catatan kehadiran</t>
-        </is>
-      </c>
-      <c r="C97" s="14" t="inlineStr">
-        <is>
-          <t>Riwayat siapa masuk kapan, durasi di ruang, status (masih di ruang / sudah keluar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="32" customHeight="1">
-      <c r="A98" s="15" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B98" s="16" t="inlineStr">
-        <is>
-          <t>Statistik kehadiran</t>
-        </is>
-      </c>
-      <c r="C98" s="17" t="inlineStr">
-        <is>
-          <t>Jumlah unik peserta, total sesi, jumlah yang masih di ruang</t>
+          <t>Cursor laser merah saat presentasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="10" customHeight="1"/>
+    <row r="97" ht="26" customHeight="1">
+      <c r="A97" s="11" t="inlineStr">
+        <is>
+          <t>6. Perekaman &amp; Pencatatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Nama Fitur</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Penjelasan</t>
         </is>
       </c>
     </row>
     <row r="99" ht="32" customHeight="1">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>Log audit</t>
+          <t>Rekaman meeting</t>
         </is>
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>Catatan semua tindakan host: kapan kunci, mute siapa, kick siapa, dll</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="10" customHeight="1"/>
-    <row r="101" ht="26" customHeight="1">
-      <c r="A101" s="11" t="inlineStr">
-        <is>
-          <t>7. Pengalaman Pengguna</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="8" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B102" s="8" t="inlineStr">
-        <is>
-          <t>Nama Fitur</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>Penjelasan</t>
+          <t>Rekam video meeting otomatis di sisi server</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="32" customHeight="1">
+      <c r="A100" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B100" s="16" t="inlineStr">
+        <is>
+          <t>Pilih layout rekaman</t>
+        </is>
+      </c>
+      <c r="C100" s="17" t="inlineStr">
+        <is>
+          <t>Pilih tampilan: grid, fokus speaker, atau solo speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="32" customHeight="1">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B101" s="13" t="inlineStr">
+        <is>
+          <t>Daftar rekaman</t>
+        </is>
+      </c>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>Lihat semua rekaman per ruang, status, dan ukuran file</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="32" customHeight="1">
+      <c r="A102" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>Unduh rekaman</t>
+        </is>
+      </c>
+      <c r="C102" s="17" t="inlineStr">
+        <is>
+          <t>Link download untuk rekaman yang sudah selesai</t>
         </is>
       </c>
     </row>
     <row r="103" ht="32" customHeight="1">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>Halaman beranda</t>
+          <t>Indikator merekam</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>Landing page profesional untuk menyambut pengguna baru</t>
+          <t>Badge merah berkedip saat rekaman aktif</t>
         </is>
       </c>
     </row>
     <row r="104" ht="32" customHeight="1">
       <c r="A104" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B104" s="16" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Banner persetujuan rekam</t>
         </is>
       </c>
       <c r="C104" s="17" t="inlineStr">
         <is>
-          <t>Halaman utama setelah login, berisi semua meeting</t>
+          <t>Notifikasi besar muncul sekali saat rekaman dimulai (untuk consent)</t>
         </is>
       </c>
     </row>
     <row r="105" ht="32" customHeight="1">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>Tema gelap &amp; terang</t>
+          <t>Catatan kehadiran</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>Toggle tema sesuai kesukaan, otomatis disimpan</t>
+          <t>Riwayat siapa masuk kapan, durasi di ruang, status (masih di ruang / sudah keluar)</t>
         </is>
       </c>
     </row>
     <row r="106" ht="32" customHeight="1">
       <c r="A106" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B106" s="16" t="inlineStr">
         <is>
-          <t>Tour onboarding</t>
+          <t>Statistik kehadiran</t>
         </is>
       </c>
       <c r="C106" s="17" t="inlineStr">
         <is>
-          <t>Panduan 5 langkah untuk pengguna pertama kali</t>
+          <t>Jumlah unik peserta, total sesi, jumlah yang masih di ruang</t>
         </is>
       </c>
     </row>
     <row r="107" ht="32" customHeight="1">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>Daftar pintasan keyboard</t>
+          <t>Log audit</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>Cheat sheet shortcut keyboard (M untuk mic, V untuk kamera, dll)</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="32" customHeight="1">
-      <c r="A108" s="15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B108" s="16" t="inlineStr">
-        <is>
-          <t>Suara efek</t>
-        </is>
-      </c>
-      <c r="C108" s="17" t="inlineStr">
-        <is>
-          <t>Notifikasi suara saat ada yang join/leave/chat/reaksi</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="32" customHeight="1">
-      <c r="A109" s="12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B109" s="13" t="inlineStr">
-        <is>
-          <t>Pengaturan suara per jenis</t>
-        </is>
-      </c>
-      <c r="C109" s="14" t="inlineStr">
-        <is>
-          <t>Bisa pilih efek mana yang nyala/mati</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="32" customHeight="1">
-      <c r="A110" s="15" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B110" s="16" t="inlineStr">
-        <is>
-          <t>Konfirmasi keluar ruang</t>
-        </is>
-      </c>
-      <c r="C110" s="17" t="inlineStr">
-        <is>
-          <t>Tanya dulu sebelum browser ditutup pas lagi meeting</t>
+          <t>Catatan semua tindakan host: kapan kunci, mute siapa, kick siapa, dll</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="10" customHeight="1"/>
+    <row r="109" ht="26" customHeight="1">
+      <c r="A109" s="11" t="inlineStr">
+        <is>
+          <t>7. Pengalaman Pengguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>Nama Fitur</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>Penjelasan</t>
         </is>
       </c>
     </row>
     <row r="111" ht="32" customHeight="1">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>Pengaturan lengkap</t>
+          <t>Halaman beranda</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
         <is>
-          <t>Halaman setting untuk akun, tampilan, audio, perangkat default</t>
+          <t>Landing page profesional untuk menyambut pengguna baru</t>
         </is>
       </c>
     </row>
     <row r="112" ht="32" customHeight="1">
       <c r="A112" s="15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B112" s="16" t="inlineStr">
         <is>
-          <t>Indikator status koneksi</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C112" s="17" t="inlineStr">
         <is>
-          <t>Tampilan kualitas internet realtime (Sangat baik / Cukup / Buruk)</t>
+          <t>Halaman utama setelah login, berisi semua meeting</t>
         </is>
       </c>
     </row>
     <row r="113" ht="32" customHeight="1">
       <c r="A113" s="12" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>Pop-up detail koneksi</t>
+          <t>Tema gelap &amp; terang</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>Klik indikator untuk lihat detail: status, jumlah peserta, identitas, room</t>
+          <t>Toggle tema sesuai kesukaan, otomatis disimpan</t>
         </is>
       </c>
     </row>
     <row r="114" ht="32" customHeight="1">
       <c r="A114" s="15" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B114" s="16" t="inlineStr">
         <is>
-          <t>Profil pribadi</t>
+          <t>Tour onboarding</t>
         </is>
       </c>
       <c r="C114" s="17" t="inlineStr">
         <is>
-          <t>Ganti nama tampilan sendiri kapan saja saat meeting</t>
+          <t>Panduan 5 langkah untuk pengguna pertama kali</t>
         </is>
       </c>
     </row>
     <row r="115" ht="32" customHeight="1">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>Status presence</t>
+          <t>Daftar pintasan keyboard</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
         <is>
-          <t>Indikator titik warna (Online / Lagi keluar / Sibuk / Jangan ganggu) di avatar setiap peserta</t>
+          <t>Cheat sheet shortcut keyboard (M untuk mic, V untuk kamera, dll)</t>
         </is>
       </c>
     </row>
     <row r="116" ht="32" customHeight="1">
       <c r="A116" s="15" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B116" s="16" t="inlineStr">
+        <is>
+          <t>Suara efek</t>
+        </is>
+      </c>
+      <c r="C116" s="17" t="inlineStr">
+        <is>
+          <t>Notifikasi suara saat ada yang join/leave/chat/reaksi</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="32" customHeight="1">
+      <c r="A117" s="12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>Pengaturan suara per jenis</t>
+        </is>
+      </c>
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>Bisa pilih efek mana yang nyala/mati</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B118" s="16" t="inlineStr">
+        <is>
+          <t>Konfirmasi keluar ruang</t>
+        </is>
+      </c>
+      <c r="C118" s="17" t="inlineStr">
+        <is>
+          <t>Tanya dulu sebelum browser ditutup pas lagi meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="32" customHeight="1">
+      <c r="A119" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>Pengaturan lengkap</t>
+        </is>
+      </c>
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>Halaman setting untuk akun, tampilan, audio, perangkat default</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="32" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B120" s="16" t="inlineStr">
+        <is>
+          <t>Indikator status koneksi</t>
+        </is>
+      </c>
+      <c r="C120" s="17" t="inlineStr">
+        <is>
+          <t>Tampilan kualitas internet realtime (Sangat baik / Cukup / Buruk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="32" customHeight="1">
+      <c r="A121" s="12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>Pop-up detail koneksi</t>
+        </is>
+      </c>
+      <c r="C121" s="14" t="inlineStr">
+        <is>
+          <t>Klik indikator untuk lihat detail: status, jumlah peserta, identitas, room</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="15" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B122" s="16" t="inlineStr">
+        <is>
+          <t>Profil pribadi</t>
+        </is>
+      </c>
+      <c r="C122" s="17" t="inlineStr">
+        <is>
+          <t>Ganti nama tampilan sendiri kapan saja saat meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="32" customHeight="1">
+      <c r="A123" s="12" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>Status presence</t>
+        </is>
+      </c>
+      <c r="C123" s="14" t="inlineStr">
+        <is>
+          <t>Indikator titik warna (Online / Lagi keluar / Sibuk / Jangan ganggu) di avatar setiap peserta</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="32" customHeight="1">
+      <c r="A124" s="15" t="inlineStr">
+        <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B116" s="16" t="inlineStr">
+      <c r="B124" s="16" t="inlineStr">
         <is>
           <t>Timer durasi meeting</t>
         </is>
       </c>
-      <c r="C116" s="17" t="inlineStr">
+      <c r="C124" s="17" t="inlineStr">
         <is>
           <t>Penghitung waktu otomatis sejak meeting dimulai</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="10" customHeight="1"/>
-    <row r="118" ht="26" customHeight="1">
-      <c r="A118" s="11" t="inlineStr">
-        <is>
-          <t>8. Multi-Bahasa</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="22" customHeight="1">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B119" s="8" t="inlineStr">
-        <is>
-          <t>Nama Fitur</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>Penjelasan</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="32" customHeight="1">
-      <c r="A120" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B120" s="13" t="inlineStr">
-        <is>
-          <t>Bahasa Indonesia</t>
-        </is>
-      </c>
-      <c r="C120" s="14" t="inlineStr">
-        <is>
-          <t>Bahasa default</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="32" customHeight="1">
-      <c r="A121" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B121" s="16" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="C121" s="17" t="inlineStr">
-        <is>
-          <t>Bahasa Inggris</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="32" customHeight="1">
-      <c r="A122" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B122" s="13" t="inlineStr">
-        <is>
-          <t>简体中文 (Mandarin)</t>
-        </is>
-      </c>
-      <c r="C122" s="14" t="inlineStr">
-        <is>
-          <t>Bahasa Mandarin Tiongkok</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="32" customHeight="1">
-      <c r="A123" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B123" s="16" t="inlineStr">
-        <is>
-          <t>Español</t>
-        </is>
-      </c>
-      <c r="C123" s="17" t="inlineStr">
-        <is>
-          <t>Bahasa Spanyol</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="32" customHeight="1">
-      <c r="A124" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B124" s="13" t="inlineStr">
-        <is>
-          <t>Pemilih bahasa</t>
-        </is>
-      </c>
-      <c r="C124" s="14" t="inlineStr">
-        <is>
-          <t>Tombol 🌐 di header untuk ganti bahasa kapan saja, otomatis disimpan</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2886,7 @@
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="11" t="inlineStr">
         <is>
-          <t>9. Keamanan &amp; Anti-Penyalahgunaan</t>
+          <t>8. Multi-Bahasa</t>
         </is>
       </c>
     </row>
@@ -2877,12 +2915,12 @@
       </c>
       <c r="B128" s="13" t="inlineStr">
         <is>
-          <t>Watermark share layar</t>
+          <t>Bahasa Indonesia</t>
         </is>
       </c>
       <c r="C128" s="14" t="inlineStr">
         <is>
-          <t>Nama dan jam viewer otomatis muncul di share layar untuk akuntabilitas</t>
+          <t>Bahasa default</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2932,12 @@
       </c>
       <c r="B129" s="16" t="inlineStr">
         <is>
-          <t>Konfirmasi keluar ruang</t>
+          <t>English</t>
         </is>
       </c>
       <c r="C129" s="17" t="inlineStr">
         <is>
-          <t>Browser tanya konfirmasi sebelum tutup tab pas meeting</t>
+          <t>Bahasa Inggris</t>
         </is>
       </c>
     </row>
@@ -2911,12 +2949,12 @@
       </c>
       <c r="B130" s="13" t="inlineStr">
         <is>
-          <t>Login wajib untuk fitur tertentu</t>
+          <t>简体中文 (Mandarin)</t>
         </is>
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>Buat ruang dan rekaman hanya untuk user terdaftar</t>
+          <t>Bahasa Mandarin Tiongkok</t>
         </is>
       </c>
     </row>
@@ -2928,27 +2966,137 @@
       </c>
       <c r="B131" s="16" t="inlineStr">
         <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="C131" s="17" t="inlineStr">
+        <is>
+          <t>Bahasa Spanyol</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="32" customHeight="1">
+      <c r="A132" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B132" s="13" t="inlineStr">
+        <is>
+          <t>Pemilih bahasa</t>
+        </is>
+      </c>
+      <c r="C132" s="14" t="inlineStr">
+        <is>
+          <t>Tombol 🌐 di header untuk ganti bahasa kapan saja, otomatis disimpan</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="10" customHeight="1"/>
+    <row r="134" ht="26" customHeight="1">
+      <c r="A134" s="11" t="inlineStr">
+        <is>
+          <t>9. Keamanan &amp; Anti-Penyalahgunaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B135" s="8" t="inlineStr">
+        <is>
+          <t>Nama Fitur</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>Penjelasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="32" customHeight="1">
+      <c r="A136" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B136" s="13" t="inlineStr">
+        <is>
+          <t>Watermark share layar</t>
+        </is>
+      </c>
+      <c r="C136" s="14" t="inlineStr">
+        <is>
+          <t>Nama dan jam viewer otomatis muncul di share layar untuk akuntabilitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="32" customHeight="1">
+      <c r="A137" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B137" s="16" t="inlineStr">
+        <is>
+          <t>Konfirmasi keluar ruang</t>
+        </is>
+      </c>
+      <c r="C137" s="17" t="inlineStr">
+        <is>
+          <t>Browser tanya konfirmasi sebelum tutup tab pas meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="32" customHeight="1">
+      <c r="A138" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B138" s="13" t="inlineStr">
+        <is>
+          <t>Login wajib untuk fitur tertentu</t>
+        </is>
+      </c>
+      <c r="C138" s="14" t="inlineStr">
+        <is>
+          <t>Buat ruang dan rekaman hanya untuk user terdaftar</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="32" customHeight="1">
+      <c r="A139" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B139" s="16" t="inlineStr">
+        <is>
           <t>Validasi domain email</t>
         </is>
       </c>
-      <c r="C131" s="17" t="inlineStr">
+      <c r="C139" s="17" t="inlineStr">
         <is>
           <t>Bisa batasi pendaftaran ke domain tertentu (untuk perusahaan)</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="10" customHeight="1"/>
+    <row r="140" ht="10" customHeight="1"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A134:C134"/>
+    <mergeCell ref="A50:C50"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A118:C118"/>
     <mergeCell ref="A126:C126"/>
-    <mergeCell ref="A89:C89"/>
+    <mergeCell ref="A97:C97"/>
+    <mergeCell ref="A109:C109"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A69:C69"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="A101:C101"/>
-    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -2962,7 +3110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2990,7 +3138,7 @@
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Prioritas 1 — Subtitle &amp; AI (Sprint 3 berikutnya)</t>
+          <t>Prioritas 1 — Subtitle &amp; AI (Sprint 3, butuh anggaran API)</t>
         </is>
       </c>
     </row>
@@ -3129,284 +3277,284 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Mode Webinar</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Speaker on stage + penonton hanya nonton &amp; chat. Cocok untuk training, kelas online, atau acara publik.</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
+    <row r="10" ht="10" customHeight="1"/>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Prioritas 2 — Mobile &amp; Distribusi (Sprint 4, tanpa biaya API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Nama Fitur</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Manfaat / Penjelasan</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Tingkat Manfaat</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Estimasi Waktu</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Aplikasi Android (.apk)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Bungkus aplikasi web jadi aplikasi Android yang bisa di-install. Teknologi Capacitor sudah disiapkan.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>2-3 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Aplikasi iOS (.ipa)</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Sama dengan Android, tapi versi iPhone/iPad. Butuh akun Apple Developer ($99/tahun).</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>2-3 hari + biaya akun</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>PWA (Install dari browser)</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Pengguna bisa 'install' aplikasi dari browser ke desktop/HP tanpa masuk app store.</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>2 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="10" customHeight="1"/>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Prioritas 2 — Penyempurnaan Chat (Sprint 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>1 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="10" customHeight="1"/>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Prioritas 3 — Persiapan Produksi (Sprint 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Nama Fitur</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Manfaat / Penjelasan</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Tingkat Manfaat</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Estimasi Waktu</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="50" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Upload file di chat</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>Kirim dokumen, gambar, atau file ke peserta lewat chat.</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>1 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="50" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Sewa server (VPS)</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Server kecil untuk menjalankan aplikasi online. Estimasi biaya: 80-150 ribu/bulan.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>1 hari + biaya bulanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>GIF picker</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="inlineStr">
-        <is>
-          <t>Sisipin GIF dari Giphy ke chat.</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>Setengah hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="50" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Daftar domain &amp; SSL</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Nama website (mis: meeting.perusahaan.com) + sertifikat keamanan HTTPS. Biaya: ~200 ribu/tahun.</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>1 hari + biaya tahunan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Reply / thread chat</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Balas pesan tertentu (quote), bukan cuma kirim balasan baru.</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>1 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="50" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>LiveKit Cloud (layanan video)</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Service untuk infrastruktur video call profesional. Versi gratis ada (~50 menit/bulan), berbayar mulai $50/bulan.</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>1 hari + biaya bulanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>Pin pesan penting</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>Tandai pesan tertentu agar muncul di atas untuk semua orang.</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
-        </is>
-      </c>
-      <c r="E17" s="15" t="inlineStr">
-        <is>
-          <t>Setengah hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="50" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Indikator 'sedang mengetik'</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Tampilkan 'Andi sedang mengetik...' di chat.</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>Setengah hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="50" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Centang 'dibaca' di DM</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>Status pesan terlihat / belum di Direct Message.</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
-        </is>
-      </c>
-      <c r="E19" s="15" t="inlineStr">
-        <is>
-          <t>1 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="10" customHeight="1"/>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Prioritas 3 — Sentuhan Sosial / Fun</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Nama Fitur</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Manfaat / Penjelasan</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Tingkat Manfaat</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Estimasi Waktu</t>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Penyimpanan rekaman (S3 / R2)</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Tempat simpan file rekaman cloud. Cloudflare R2: 10 GB gratis. AWS S3 / Backblaze juga opsi.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Setengah hari + biaya bulanan</t>
         </is>
       </c>
     </row>
     <row r="23" ht="50" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Soundboard</t>
+          <t>Monitoring sistem</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Tombol untuk mainkan efek suara (tepuk tangan, drum roll) ke semua peserta. Discord-style.</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
+          <t>Pantau apakah aplikasi nyala atau down. Pakai Uptime Kuma (gratis).</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Sedang</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -3418,335 +3566,335 @@
     <row r="24" ht="50" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>Mini games dalam meeting</t>
+          <t>Pelacakan error (Sentry)</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>Game seperti tebak-tebakan, kuis ringan untuk ice breaker.</t>
-        </is>
-      </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
+          <t>Otomatis catat error yang terjadi di aplikasi untuk perbaikan cepat. Versi gratis cukup.</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Sedang</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>2-3 hari</t>
+          <t>Setengah hari</t>
         </is>
       </c>
     </row>
     <row r="25" ht="50" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
+          <t>Halaman bantuan / FAQ</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Halaman dokumentasi user (cara buat meeting, ganti password, dll).</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>1-2 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Lupa password / verifikasi email</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Lupa password lewat email, verifikasi email saat daftar. Butuh integrasi pengiriman email.</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>1 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="10" customHeight="1"/>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Prioritas 4 — Sentuhan Sosial (opsional, bisa dikerjakan sela)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Nama Fitur</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Manfaat / Penjelasan</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Tingkat Manfaat</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Estimasi Waktu</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Mini games dalam meeting</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Game seperti tebak-tebakan, kuis ringan untuk ice breaker.</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Rendah</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>2-3 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
           <t>Threshold suara otomatis</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>Mic otomatis aktif hanya kalau ada suara di atas batas tertentu.</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Rendah</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>Setengah hari</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="10" customHeight="1"/>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Prioritas 4 — Fitur Perusahaan (Enterprise)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="32" ht="10" customHeight="1"/>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Prioritas 5 — Fitur Perusahaan (Enterprise, opsional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Nama Fitur</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>Manfaat / Penjelasan</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>Tingkat Manfaat</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>Estimasi Waktu</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="50" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Dial-in via telepon</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>Peserta bisa join meeting lewat panggilan telepon biasa (tanpa internet). Butuh Twilio, biaya per menit.</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>Rendah</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>3-5 hari + biaya bulanan</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="50" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>Login dengan Google / Microsoft Workspace (SSO)</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>Karyawan bisa login pakai akun perusahaan langsung. Penting untuk customer enterprise.</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D36" s="18" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E36" s="15" t="inlineStr">
         <is>
           <t>2-3 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="50" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Enkripsi end-to-end (E2EE)</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="inlineStr">
-        <is>
-          <t>Video dienkripsi sehingga bahkan server tidak bisa lihat. Penting untuk industri sensitif (hukum, medis).</t>
-        </is>
-      </c>
-      <c r="D31" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>2 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="50" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B32" s="16" t="inlineStr">
-        <is>
-          <t>Mode 'Together' (avatar virtual)</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>Semua peserta tampil duduk bersebelahan di ruang virtual 3D (Microsoft Teams-style).</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>1 minggu</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="50" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Companion mode</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="inlineStr">
-        <is>
-          <t>Device kedua (HP) join meeting tanpa audio/video, hanya untuk chat dan reaksi.</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>Rendah</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>1 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="10" customHeight="1"/>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>Prioritas 5 — Mobile &amp; Distribusi (Sprint 4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Nama Fitur</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Manfaat / Penjelasan</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Tingkat Manfaat</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Estimasi Waktu</t>
         </is>
       </c>
     </row>
     <row r="37" ht="50" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Aplikasi Android (.apk)</t>
+          <t>Enkripsi end-to-end (E2EE)</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
         <is>
-          <t>Bungkus aplikasi web jadi aplikasi Android yang bisa di-install. Teknologi Capacitor sudah disiapkan.</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
+          <t>Video dienkripsi sehingga bahkan server tidak bisa lihat. Penting untuk industri sensitif (hukum, medis).</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>Sedang</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>2-3 hari</t>
+          <t>2 hari</t>
         </is>
       </c>
     </row>
     <row r="38" ht="50" customHeight="1">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>Aplikasi iOS (.ipa)</t>
+          <t>Mode 'Together' (avatar virtual)</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>Sama dengan Android, tapi versi iPhone/iPad. Butuh akun Apple Developer ($99/tahun).</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
+          <t>Semua peserta tampil duduk bersebelahan di ruang virtual 3D (Microsoft Teams-style).</t>
+        </is>
+      </c>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>Rendah</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>2-3 hari + biaya akun</t>
+          <t>1 minggu</t>
         </is>
       </c>
     </row>
     <row r="39" ht="50" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>PWA (Install dari browser)</t>
+          <t>Companion mode</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
         <is>
-          <t>Pengguna bisa 'install' aplikasi dari browser ke desktop/HP tanpa masuk app store.</t>
-        </is>
-      </c>
-      <c r="D39" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
+          <t>Device kedua (HP) join meeting tanpa audio/video, hanya untuk chat dan reaksi.</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>Rendah</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
@@ -3756,282 +3904,30 @@
       </c>
     </row>
     <row r="40" ht="10" customHeight="1"/>
-    <row r="41" ht="26" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>Prioritas 6 — Persiapan Produksi (Sprint 6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Nama Fitur</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Manfaat / Penjelasan</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Tingkat Manfaat</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Estimasi Waktu</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="50" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>Sewa server (VPS)</t>
-        </is>
-      </c>
-      <c r="C43" s="14" t="inlineStr">
-        <is>
-          <t>Server kecil untuk menjalankan aplikasi online. Estimasi biaya: 80-150 ribu/bulan.</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>1 hari + biaya bulanan</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="50" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>Daftar domain &amp; SSL</t>
-        </is>
-      </c>
-      <c r="C44" s="17" t="inlineStr">
-        <is>
-          <t>Nama website (mis: meeting.perusahaan.com) + sertifikat keamanan HTTPS. Biaya: ~200 ribu/tahun.</t>
-        </is>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>1 hari + biaya tahunan</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="50" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>LiveKit Cloud (layanan video)</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="inlineStr">
-        <is>
-          <t>Service untuk infrastruktur video call profesional. Versi gratis ada (~50 menit/bulan), berbayar mulai $50/bulan.</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>1 hari + biaya bulanan</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="50" customHeight="1">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>Penyimpanan rekaman (S3 / R2)</t>
-        </is>
-      </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>Tempat simpan file rekaman cloud. Cloudflare R2: 10 GB gratis. AWS S3 / Backblaze juga opsi.</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
-        </is>
-      </c>
-      <c r="E46" s="15" t="inlineStr">
-        <is>
-          <t>Setengah hari + biaya bulanan</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="50" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>Monitoring sistem</t>
-        </is>
-      </c>
-      <c r="C47" s="14" t="inlineStr">
-        <is>
-          <t>Pantau apakah aplikasi nyala atau down. Pakai Uptime Kuma (gratis).</t>
-        </is>
-      </c>
-      <c r="D47" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>Setengah hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="50" customHeight="1">
-      <c r="A48" s="15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>Pelacakan error (Sentry)</t>
-        </is>
-      </c>
-      <c r="C48" s="17" t="inlineStr">
-        <is>
-          <t>Otomatis catat error yang terjadi di aplikasi untuk perbaikan cepat. Versi gratis cukup.</t>
-        </is>
-      </c>
-      <c r="D48" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
-      </c>
-      <c r="E48" s="15" t="inlineStr">
-        <is>
-          <t>Setengah hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="50" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>Halaman bantuan / FAQ</t>
-        </is>
-      </c>
-      <c r="C49" s="14" t="inlineStr">
-        <is>
-          <t>Halaman dokumentasi user (cara buat meeting, ganti password, dll).</t>
-        </is>
-      </c>
-      <c r="D49" s="18" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>1-2 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="50" customHeight="1">
-      <c r="A50" s="15" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B50" s="16" t="inlineStr">
-        <is>
-          <t>Lupa password / verifikasi email</t>
-        </is>
-      </c>
-      <c r="C50" s="17" t="inlineStr">
-        <is>
-          <t>Lupa password lewat email, verifikasi email saat daftar. Butuh integrasi pengiriman email.</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
-        <is>
-          <t>Tinggi</t>
-        </is>
-      </c>
-      <c r="E50" s="15" t="inlineStr">
-        <is>
-          <t>1 hari</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="10" customHeight="1"/>
-    <row r="53" ht="30" customHeight="1">
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Tingkat Manfaat</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>Tinggi = sangat berdampak ke pengalaman pengguna   ·   Sedang = nice-to-have   ·   Rendah = pelengkap</t>
         </is>
       </c>
-      <c r="D53" s="20" t="n"/>
-      <c r="E53" s="21" t="n"/>
+      <c r="D42" s="20" t="n"/>
+      <c r="E42" s="21" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A12:E12"/>
+  <mergeCells count="8">
+    <mergeCell ref="C42:E42"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A17:E17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4906,26 +4802,26 @@
     </row>
     <row r="38" ht="12" customHeight="1"/>
     <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 5 — Penyempurnaan Chat &amp; Sosial</t>
-        </is>
-      </c>
-      <c r="D39" s="26" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 5 — Penyempurnaan Chat &amp; Webinar ✓</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
         <is>
           <t>Durasi: 1 minggu</t>
         </is>
       </c>
-      <c r="F39" s="26" t="inlineStr">
-        <is>
-          <t>BELUM</t>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>Fitur tambahan untuk meningkatkan kualitas komunikasi dan engagement.</t>
+          <t>Selesai. Chat sekelas Slack (file, reply, pin, typing, read receipts, GIF, soundboard) + Mode Webinar untuk training internal.</t>
         </is>
       </c>
     </row>
@@ -4974,7 +4870,7 @@
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>Upload file di chat (PDF, gambar, dokumen)</t>
+          <t>Upload file di chat (PDF, gambar, dokumen Office) sampai 10 MB</t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr">
@@ -4987,9 +4883,9 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="F42" s="10" t="inlineStr">
-        <is>
-          <t>Belum</t>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -5006,12 +4902,12 @@
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>Reply / thread di chat + Pin pesan penting</t>
+          <t>Reply/quote pesan + Pin pesan penting (host-only, sticky banner)</t>
         </is>
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
-          <t>Diskusi terstruktur, info penting tidak hilang</t>
+          <t>Diskusi terstruktur, info penting tidak hilang di scroll</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
@@ -5019,9 +4915,9 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
-        <is>
-          <t>Belum</t>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -5038,7 +4934,7 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>Indikator 'sedang mengetik' + Centang 'dibaca' di DM</t>
+          <t>Indikator 'sedang mengetik' + Centang ✓ / ✓✓ di DM</t>
         </is>
       </c>
       <c r="D44" s="14" t="inlineStr">
@@ -5051,9 +4947,9 @@
           <t>Rendah</t>
         </is>
       </c>
-      <c r="F44" s="10" t="inlineStr">
-        <is>
-          <t>Belum</t>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -5070,7 +4966,7 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>GIF picker + Soundboard (fun elements)</t>
+          <t>GIF picker (Giphy) + Soundboard (8 preset efek suara)</t>
         </is>
       </c>
       <c r="D45" s="17" t="inlineStr">
@@ -5083,9 +4979,9 @@
           <t>Rendah</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
-        <is>
-          <t>Belum</t>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -5102,12 +4998,12 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>Mode Webinar (presenter + audience watch-only)</t>
+          <t>Mode Webinar (presenter + audience watch-only, LiveKit token grant)</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>Cocok untuk training internal</t>
+          <t>Cocok untuk training internal, kelas online</t>
         </is>
       </c>
       <c r="E46" s="18" t="inlineStr">
@@ -5115,9 +5011,9 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="F46" s="10" t="inlineStr">
-        <is>
-          <t>Belum</t>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -5346,15 +5242,20 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="150" customHeight="1">
+    <row r="59" ht="200" customHeight="1">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>1. Sprint 1 (Penyempurnaan Cepat) dan Sprint 2 (Fitur Wow Visual) sudah SELESAI per 2026-06-20.
-2. Sisa 4 sprint = 4 minggu kerja untuk menyelesaikan semua roadmap.
-3. Sprint 3 (AI) dan Sprint 6 (Produksi) butuh keputusan anggaran karena ada biaya bulanan: API AI (~Rp 200-500 ribu/bulan), server (~Rp 80-150 ribu/bulan), layanan video (~Rp 800 ribu/bulan).
-4. Sprint 4 (Mobile) dan Sprint 5 (Chat) bisa dikerjakan tanpa biaya tambahan.
-5. Urutan sprint bisa dirubah sesuai prioritas bisnis. Misalnya, kalau target utama internal pakai dulu, Sprint 6 (Produksi) bisa ditunda ke akhir.
-6. Estimasi waktu mengasumsikan tidak ada blocker besar. Buffer 1-2 hari per sprint untuk testing dan polish.</t>
+          <t>1. Sprint 1, 2, dan 5 sudah SELESAI. 50% dari roadmap sudah tuntas.
+2. Sisa 3 sprint = ~3 minggu kerja untuk menyelesaikan semua roadmap.
+3. Sprint 3 (AI) dan Sprint 6 (Produksi) butuh keputusan anggaran karena ada biaya bulanan:
+   • API AI ~Rp 200-500 ribu/bulan (Whisper / Deepgram)
+   • Server VPS ~Rp 80-150 ribu/bulan
+   • Layanan video (LiveKit Cloud) ~Rp 800 ribu/bulan setelah free tier
+4. Sprint 4 (Mobile) bisa dikerjakan tanpa biaya tambahan (Android gratis; iOS butuh akun Apple Dev $99/tahun).
+5. Rekomendasi urutan berikut:
+   • Sprint 4 (Mobile) — hasilnya paling kelihatan, gratis, langsung bisa demo di HP
+   • Sprint 6 (Produksi) — biar aplikasi bisa dipakai online
+   • Sprint 3 (AI) — kalau anggaran keluar, ini fitur pembeda utama</t>
         </is>
       </c>
       <c r="B59" s="20" t="n"/>

</xml_diff>